<commit_message>
axozee: plano de corte passa a identificar a malha por nome e cor
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YJvJ7mkA9K2C8Ac53hAWfB
</commit_message>
<xml_diff>
--- a/axozee/corte/AXOZEE-Plano-de-Corte-v1.xlsx
+++ b/axozee/corte/AXOZEE-Plano-de-Corte-v1.xlsx
@@ -15,7 +15,7 @@
     <sheet name="COMO USAR" sheetId="5" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">MALHAS!$A$1:$M$9</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">MALHAS!$A$1:$N$9</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="_xlnm.Print_Area" vbProcedure="false">MODELAGENS!$A$1:$G$8</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">PAINEL!$A$1:$L$52</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'PLANO DE CORTE'!$A$1:$N$23</definedName>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="144">
   <si>
     <t xml:space="preserve">AXOZEE  ·  PAINEL DE CORTE</t>
   </si>
@@ -237,112 +237,121 @@
     <t xml:space="preserve">CP-01</t>
   </si>
   <si>
+    <t xml:space="preserve">Algodão Pima Preta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Axozee Slim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CP-02</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CP-03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CP-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CP-05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Axozee Over</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CP-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CP-07</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CP-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CP-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peruana Off White</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CP-10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CP-11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CP-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CP-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CP-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CP-15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CP-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MALHAS  ·  ESTOQUE E RENDIMENTO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linhas em amarelo são preenchidas por você. O resto é calculado.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Código</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kg disponível</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rendimento previsto (pç/kg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capacidade prevista (pç)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peças planejadas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kg previsto p/ o plano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peças cortadas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kg real consumido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rendimento real (pç/kg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desvio vs previsto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Saldo de malha (kg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nome usado no plano de corte</t>
+  </si>
+  <si>
     <t xml:space="preserve">M1</t>
   </si>
   <si>
-    <t xml:space="preserve">Axozee Slim</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CP-02</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CP-03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CP-04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CP-05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Axozee Over</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CP-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CP-07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CP-08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CP-09</t>
+    <t xml:space="preserve">Algodão Pima</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preta</t>
   </si>
   <si>
     <t xml:space="preserve">M2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CP-10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CP-11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CP-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CP-13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CP-14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CP-15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CP-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MALHAS  ·  ESTOQUE E RENDIMENTO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Linhas em amarelo são preenchidas por você. O resto é calculado.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Código</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kg disponível</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rendimento previsto (pç/kg)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Capacidade prevista (pç)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peças planejadas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kg previsto p/ o plano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peças cortadas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kg real consumido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rendimento real (pç/kg)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Desvio vs previsto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Saldo de malha (kg)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Algodão Pima</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preta</t>
   </si>
   <si>
     <t xml:space="preserve">Peruana</t>
@@ -514,7 +523,7 @@
     <numFmt numFmtId="169" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="170" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="37">
+  <fonts count="38">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -713,6 +722,14 @@
     <font>
       <b val="true"/>
       <sz val="10"/>
+      <color rgb="FF555C3A"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
       <color rgb="FFEEE7D6"/>
       <name val="Arial"/>
       <family val="0"/>
@@ -918,7 +935,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1091,11 +1108,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="27" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="27" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="170" fontId="27" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="170" fontId="28" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="28" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1107,59 +1128,59 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="28" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="29" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="30" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="31" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="30" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="30" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="30" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="27" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="28" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="32" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="33" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="33" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="34" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="34" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="35" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="35" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="36" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="36" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="37" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="29" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="30" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1677,11 +1698,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="1818711"/>
-        <c:axId val="9286731"/>
+        <c:axId val="3947435"/>
+        <c:axId val="21192318"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1818711"/>
+        <c:axId val="3947435"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1747,7 +1768,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9286731"/>
+        <c:crossAx val="21192318"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1755,7 +1776,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="9286731"/>
+        <c:axId val="21192318"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1831,7 +1852,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1818711"/>
+        <c:crossAx val="3947435"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2086,11 +2107,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="15603678"/>
-        <c:axId val="5813754"/>
+        <c:axId val="89749192"/>
+        <c:axId val="61229551"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="15603678"/>
+        <c:axId val="89749192"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2122,7 +2143,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="5813754"/>
+        <c:crossAx val="61229551"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2130,7 +2151,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="5813754"/>
+        <c:axId val="61229551"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2172,7 +2193,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="15603678"/>
+        <c:crossAx val="89749192"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3368,7 +3389,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{FE6A9B87-BDFB-4450-9B88-90A4BA297C66}</x14:id>
+          <x14:id>{A93FF82A-F6F9-4736-B4B0-747AAEF278CA}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3382,7 +3403,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2E592063-6949-48E0-84A7-6358ABFFD067}</x14:id>
+          <x14:id>{77F847FF-57A6-4217-A83A-B9FF6BE8DB10}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -3421,7 +3442,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{FE6A9B87-BDFB-4450-9B88-90A4BA297C66}">
+          <x14:cfRule type="dataBar" id="{A93FF82A-F6F9-4736-B4B0-747AAEF278CA}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -3436,7 +3457,7 @@
           <xm:sqref>E13:E14</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2E592063-6949-48E0-84A7-6358ABFFD067}">
+          <x14:cfRule type="dataBar" id="{77F847FF-57A6-4217-A83A-B9FF6BE8DB10}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -3466,7 +3487,7 @@
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="21"/>
@@ -3476,8 +3497,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="22"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3642,7 +3663,7 @@
         <v>PENDENTE</v>
       </c>
       <c r="K7" s="14" t="n">
-        <f aca="false">IFERROR(F7/INDEX(MALHAS!$E$5:$E$6,MATCH($B7,MALHAS!$A$5:$A$6,0)),0)</f>
+        <f aca="false">IFERROR(F7/INDEX(MALHAS!$E$5:$E$6,MATCH($B7,MALHAS!$N$5:$N$6,0)),0)</f>
         <v>1</v>
       </c>
       <c r="L7" s="30"/>
@@ -3685,7 +3706,7 @@
         <v>PENDENTE</v>
       </c>
       <c r="K8" s="14" t="n">
-        <f aca="false">IFERROR(F8/INDEX(MALHAS!$E$5:$E$6,MATCH($B8,MALHAS!$A$5:$A$6,0)),0)</f>
+        <f aca="false">IFERROR(F8/INDEX(MALHAS!$E$5:$E$6,MATCH($B8,MALHAS!$N$5:$N$6,0)),0)</f>
         <v>2</v>
       </c>
       <c r="L8" s="30"/>
@@ -3728,7 +3749,7 @@
         <v>PENDENTE</v>
       </c>
       <c r="K9" s="14" t="n">
-        <f aca="false">IFERROR(F9/INDEX(MALHAS!$E$5:$E$6,MATCH($B9,MALHAS!$A$5:$A$6,0)),0)</f>
+        <f aca="false">IFERROR(F9/INDEX(MALHAS!$E$5:$E$6,MATCH($B9,MALHAS!$N$5:$N$6,0)),0)</f>
         <v>4</v>
       </c>
       <c r="L9" s="30"/>
@@ -3771,7 +3792,7 @@
         <v>PENDENTE</v>
       </c>
       <c r="K10" s="14" t="n">
-        <f aca="false">IFERROR(F10/INDEX(MALHAS!$E$5:$E$6,MATCH($B10,MALHAS!$A$5:$A$6,0)),0)</f>
+        <f aca="false">IFERROR(F10/INDEX(MALHAS!$E$5:$E$6,MATCH($B10,MALHAS!$N$5:$N$6,0)),0)</f>
         <v>3</v>
       </c>
       <c r="L10" s="30"/>
@@ -3814,7 +3835,7 @@
         <v>SEM PLANO</v>
       </c>
       <c r="K11" s="14" t="n">
-        <f aca="false">IFERROR(F11/INDEX(MALHAS!$E$5:$E$6,MATCH($B11,MALHAS!$A$5:$A$6,0)),0)</f>
+        <f aca="false">IFERROR(F11/INDEX(MALHAS!$E$5:$E$6,MATCH($B11,MALHAS!$N$5:$N$6,0)),0)</f>
         <v>0</v>
       </c>
       <c r="L11" s="30"/>
@@ -3857,7 +3878,7 @@
         <v>SEM PLANO</v>
       </c>
       <c r="K12" s="14" t="n">
-        <f aca="false">IFERROR(F12/INDEX(MALHAS!$E$5:$E$6,MATCH($B12,MALHAS!$A$5:$A$6,0)),0)</f>
+        <f aca="false">IFERROR(F12/INDEX(MALHAS!$E$5:$E$6,MATCH($B12,MALHAS!$N$5:$N$6,0)),0)</f>
         <v>0</v>
       </c>
       <c r="L12" s="30"/>
@@ -3900,7 +3921,7 @@
         <v>PENDENTE</v>
       </c>
       <c r="K13" s="14" t="n">
-        <f aca="false">IFERROR(F13/INDEX(MALHAS!$E$5:$E$6,MATCH($B13,MALHAS!$A$5:$A$6,0)),0)</f>
+        <f aca="false">IFERROR(F13/INDEX(MALHAS!$E$5:$E$6,MATCH($B13,MALHAS!$N$5:$N$6,0)),0)</f>
         <v>2</v>
       </c>
       <c r="L13" s="30"/>
@@ -3943,7 +3964,7 @@
         <v>SEM PLANO</v>
       </c>
       <c r="K14" s="14" t="n">
-        <f aca="false">IFERROR(F14/INDEX(MALHAS!$E$5:$E$6,MATCH($B14,MALHAS!$A$5:$A$6,0)),0)</f>
+        <f aca="false">IFERROR(F14/INDEX(MALHAS!$E$5:$E$6,MATCH($B14,MALHAS!$N$5:$N$6,0)),0)</f>
         <v>0</v>
       </c>
       <c r="L14" s="30"/>
@@ -3986,7 +4007,7 @@
         <v>SEM PLANO</v>
       </c>
       <c r="K15" s="14" t="n">
-        <f aca="false">IFERROR(F15/INDEX(MALHAS!$E$5:$E$6,MATCH($B15,MALHAS!$A$5:$A$6,0)),0)</f>
+        <f aca="false">IFERROR(F15/INDEX(MALHAS!$E$5:$E$6,MATCH($B15,MALHAS!$N$5:$N$6,0)),0)</f>
         <v>0</v>
       </c>
       <c r="L15" s="30"/>
@@ -4029,7 +4050,7 @@
         <v>SEM PLANO</v>
       </c>
       <c r="K16" s="14" t="n">
-        <f aca="false">IFERROR(F16/INDEX(MALHAS!$E$5:$E$6,MATCH($B16,MALHAS!$A$5:$A$6,0)),0)</f>
+        <f aca="false">IFERROR(F16/INDEX(MALHAS!$E$5:$E$6,MATCH($B16,MALHAS!$N$5:$N$6,0)),0)</f>
         <v>0</v>
       </c>
       <c r="L16" s="30"/>
@@ -4072,7 +4093,7 @@
         <v>PENDENTE</v>
       </c>
       <c r="K17" s="14" t="n">
-        <f aca="false">IFERROR(F17/INDEX(MALHAS!$E$5:$E$6,MATCH($B17,MALHAS!$A$5:$A$6,0)),0)</f>
+        <f aca="false">IFERROR(F17/INDEX(MALHAS!$E$5:$E$6,MATCH($B17,MALHAS!$N$5:$N$6,0)),0)</f>
         <v>1.11111111111111</v>
       </c>
       <c r="L17" s="30"/>
@@ -4115,7 +4136,7 @@
         <v>PENDENTE</v>
       </c>
       <c r="K18" s="14" t="n">
-        <f aca="false">IFERROR(F18/INDEX(MALHAS!$E$5:$E$6,MATCH($B18,MALHAS!$A$5:$A$6,0)),0)</f>
+        <f aca="false">IFERROR(F18/INDEX(MALHAS!$E$5:$E$6,MATCH($B18,MALHAS!$N$5:$N$6,0)),0)</f>
         <v>1.11111111111111</v>
       </c>
       <c r="L18" s="30"/>
@@ -4158,7 +4179,7 @@
         <v>PENDENTE</v>
       </c>
       <c r="K19" s="14" t="n">
-        <f aca="false">IFERROR(F19/INDEX(MALHAS!$E$5:$E$6,MATCH($B19,MALHAS!$A$5:$A$6,0)),0)</f>
+        <f aca="false">IFERROR(F19/INDEX(MALHAS!$E$5:$E$6,MATCH($B19,MALHAS!$N$5:$N$6,0)),0)</f>
         <v>2.22222222222222</v>
       </c>
       <c r="L19" s="30"/>
@@ -4201,7 +4222,7 @@
         <v>PENDENTE</v>
       </c>
       <c r="K20" s="14" t="n">
-        <f aca="false">IFERROR(F20/INDEX(MALHAS!$E$5:$E$6,MATCH($B20,MALHAS!$A$5:$A$6,0)),0)</f>
+        <f aca="false">IFERROR(F20/INDEX(MALHAS!$E$5:$E$6,MATCH($B20,MALHAS!$N$5:$N$6,0)),0)</f>
         <v>4.44444444444445</v>
       </c>
       <c r="L20" s="30"/>
@@ -4244,7 +4265,7 @@
         <v>PENDENTE</v>
       </c>
       <c r="K21" s="14" t="n">
-        <f aca="false">IFERROR(F21/INDEX(MALHAS!$E$5:$E$6,MATCH($B21,MALHAS!$A$5:$A$6,0)),0)</f>
+        <f aca="false">IFERROR(F21/INDEX(MALHAS!$E$5:$E$6,MATCH($B21,MALHAS!$N$5:$N$6,0)),0)</f>
         <v>4.44444444444445</v>
       </c>
       <c r="L21" s="30"/>
@@ -4287,7 +4308,7 @@
         <v>PENDENTE</v>
       </c>
       <c r="K22" s="14" t="n">
-        <f aca="false">IFERROR(F22/INDEX(MALHAS!$E$5:$E$6,MATCH($B22,MALHAS!$A$5:$A$6,0)),0)</f>
+        <f aca="false">IFERROR(F22/INDEX(MALHAS!$E$5:$E$6,MATCH($B22,MALHAS!$N$5:$N$6,0)),0)</f>
         <v>4.44444444444445</v>
       </c>
       <c r="L22" s="30"/>
@@ -4369,7 +4390,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{D4CD8151-BB20-48A6-8A2A-424066CA1BC2}</x14:id>
+          <x14:id>{00A3841A-E118-45C6-A96C-4C2BA9342AE5}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -4380,8 +4401,8 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="5">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" prompt="M1 = Algodão Pima Preta · M2 = Peruana Off White" promptTitle="Malha" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B7:B22" type="list">
-      <formula1>"M1,M2"</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" prompt="Escolha a malha. Para incluir outra, cadastre na aba MALHAS." promptTitle="Malha" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B7:B22" type="list">
+      <formula1>"Algodão Pima Preta,Peruana Off White"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C7:C22" type="list">
@@ -4414,7 +4435,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{D4CD8151-BB20-48A6-8A2A-424066CA1BC2}">
+          <x14:cfRule type="dataBar" id="{00A3841A-E118-45C6-A96C-4C2BA9342AE5}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -4440,11 +4461,11 @@
     <tabColor rgb="FFC45D36"/>
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:N9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
@@ -4454,6 +4475,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4472,6 +4494,7 @@
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
@@ -4489,6 +4512,7 @@
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
@@ -4530,16 +4554,19 @@
       <c r="M4" s="10" t="s">
         <v>86</v>
       </c>
+      <c r="N4" s="10" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="36" t="s">
-        <v>53</v>
+        <v>88</v>
       </c>
       <c r="B5" s="37" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C5" s="37" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D5" s="38" t="n">
         <v>12</v>
@@ -4552,7 +4579,7 @@
         <v>60</v>
       </c>
       <c r="G5" s="39" t="n">
-        <f aca="false">SUMIFS('PLANO DE CORTE'!$F$7:$F$22,'PLANO DE CORTE'!$B$7:$B$22,$A5)</f>
+        <f aca="false">SUMIFS('PLANO DE CORTE'!$F$7:$F$22,'PLANO DE CORTE'!$B$7:$B$22,$N5)</f>
         <v>60</v>
       </c>
       <c r="H5" s="39" t="n">
@@ -4560,7 +4587,7 @@
         <v>12</v>
       </c>
       <c r="I5" s="39" t="n">
-        <f aca="false">SUMIFS('PLANO DE CORTE'!$G$7:$G$22,'PLANO DE CORTE'!$B$7:$B$22,$A5)</f>
+        <f aca="false">SUMIFS('PLANO DE CORTE'!$G$7:$G$22,'PLANO DE CORTE'!$B$7:$B$22,$N5)</f>
         <v>0</v>
       </c>
       <c r="J5" s="40"/>
@@ -4576,16 +4603,20 @@
         <f aca="false">D5-IF(J5=0,H5,J5)</f>
         <v>0</v>
       </c>
+      <c r="N5" s="43" t="str">
+        <f aca="false">B5&amp;" "&amp;C5</f>
+        <v>Algodão Pima Preta</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="36" t="s">
-        <v>64</v>
+        <v>91</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C6" s="37" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="D6" s="38" t="n">
         <v>18</v>
@@ -4598,7 +4629,7 @@
         <v>81</v>
       </c>
       <c r="G6" s="39" t="n">
-        <f aca="false">SUMIFS('PLANO DE CORTE'!$F$7:$F$22,'PLANO DE CORTE'!$B$7:$B$22,$A6)</f>
+        <f aca="false">SUMIFS('PLANO DE CORTE'!$F$7:$F$22,'PLANO DE CORTE'!$B$7:$B$22,$N6)</f>
         <v>80</v>
       </c>
       <c r="H6" s="39" t="n">
@@ -4606,7 +4637,7 @@
         <v>17.7777777777778</v>
       </c>
       <c r="I6" s="39" t="n">
-        <f aca="false">SUMIFS('PLANO DE CORTE'!$G$7:$G$22,'PLANO DE CORTE'!$B$7:$B$22,$A6)</f>
+        <f aca="false">SUMIFS('PLANO DE CORTE'!$G$7:$G$22,'PLANO DE CORTE'!$B$7:$B$22,$N6)</f>
         <v>0</v>
       </c>
       <c r="J6" s="40"/>
@@ -4622,51 +4653,56 @@
         <f aca="false">D6-IF(J6=0,H6,J6)</f>
         <v>0.222222222222221</v>
       </c>
+      <c r="N6" s="43" t="str">
+        <f aca="false">B6&amp;" "&amp;C6</f>
+        <v>Peruana Off White</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="43" t="s">
+      <c r="A7" s="44" t="s">
         <v>72</v>
       </c>
-      <c r="B7" s="43"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="44" t="n">
+      <c r="B7" s="44"/>
+      <c r="C7" s="44"/>
+      <c r="D7" s="45" t="n">
         <f aca="false">SUM(D5:D6)</f>
         <v>30</v>
       </c>
-      <c r="E7" s="44"/>
-      <c r="F7" s="44" t="n">
+      <c r="E7" s="45"/>
+      <c r="F7" s="45" t="n">
         <f aca="false">SUM(F5:F6)</f>
         <v>141</v>
       </c>
-      <c r="G7" s="44" t="n">
+      <c r="G7" s="45" t="n">
         <f aca="false">SUM(G5:G6)</f>
         <v>140</v>
       </c>
-      <c r="H7" s="44" t="n">
+      <c r="H7" s="45" t="n">
         <f aca="false">SUM(H5:H6)</f>
         <v>29.7777777777778</v>
       </c>
-      <c r="I7" s="44" t="n">
+      <c r="I7" s="45" t="n">
         <f aca="false">SUM(I5:I6)</f>
         <v>0</v>
       </c>
-      <c r="J7" s="44" t="n">
+      <c r="J7" s="45" t="n">
         <f aca="false">SUM(J5:J6)</f>
         <v>0</v>
       </c>
-      <c r="K7" s="44" t="n">
+      <c r="K7" s="45" t="n">
         <f aca="false">IFERROR(I7/J7,0)</f>
         <v>0</v>
       </c>
-      <c r="L7" s="44"/>
-      <c r="M7" s="44" t="n">
+      <c r="L7" s="45"/>
+      <c r="M7" s="45" t="n">
         <f aca="false">SUM(M5:M6)</f>
         <v>0.222222222222221</v>
       </c>
+      <c r="N7" s="45"/>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="18" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B9" s="18"/>
       <c r="C9" s="18"/>
@@ -4680,13 +4716,14 @@
       <c r="K9" s="18"/>
       <c r="L9" s="18"/>
       <c r="M9" s="18"/>
+      <c r="N9" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A2:N2"/>
     <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A9:M9"/>
+    <mergeCell ref="A9:N9"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="false"/>
   <pageMargins left="0.3" right="0.3" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4717,7 +4754,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4728,7 +4765,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4742,13 +4779,13 @@
         <v>18</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="E4" s="10" t="s">
         <v>80</v>
@@ -4757,71 +4794,71 @@
         <v>82</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="45" t="s">
+      <c r="A5" s="46" t="s">
         <v>54</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C5" s="37" t="s">
-        <v>99</v>
-      </c>
-      <c r="D5" s="46" t="s">
-        <v>100</v>
-      </c>
-      <c r="E5" s="47" t="n">
+        <v>102</v>
+      </c>
+      <c r="D5" s="47" t="s">
+        <v>103</v>
+      </c>
+      <c r="E5" s="48" t="n">
         <f aca="false">SUMIFS('PLANO DE CORTE'!$F$7:$F$22,'PLANO DE CORTE'!$C$7:$C$22,$A5)</f>
         <v>60</v>
       </c>
-      <c r="F5" s="47" t="n">
+      <c r="F5" s="48" t="n">
         <f aca="false">SUMIFS('PLANO DE CORTE'!$G$7:$G$22,'PLANO DE CORTE'!$C$7:$C$22,$A5)</f>
         <v>0</v>
       </c>
-      <c r="G5" s="47" t="n">
+      <c r="G5" s="48" t="n">
         <f aca="false">IF($B5="SIM",E5,0)</f>
         <v>60</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="45" t="s">
+      <c r="A6" s="46" t="s">
         <v>59</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C6" s="37" t="s">
-        <v>102</v>
-      </c>
-      <c r="D6" s="46" t="s">
-        <v>103</v>
-      </c>
-      <c r="E6" s="47" t="n">
+        <v>105</v>
+      </c>
+      <c r="D6" s="47" t="s">
+        <v>106</v>
+      </c>
+      <c r="E6" s="48" t="n">
         <f aca="false">SUMIFS('PLANO DE CORTE'!$F$7:$F$22,'PLANO DE CORTE'!$C$7:$C$22,$A6)</f>
         <v>80</v>
       </c>
-      <c r="F6" s="47" t="n">
+      <c r="F6" s="48" t="n">
         <f aca="false">SUMIFS('PLANO DE CORTE'!$G$7:$G$22,'PLANO DE CORTE'!$C$7:$C$22,$A6)</f>
         <v>0</v>
       </c>
-      <c r="G6" s="47" t="n">
+      <c r="G6" s="48" t="n">
         <f aca="false">IF($B6="SIM",E6,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="48" t="s">
-        <v>104</v>
-      </c>
-      <c r="B8" s="48"/>
-      <c r="C8" s="48"/>
-      <c r="D8" s="48"/>
-      <c r="E8" s="48"/>
-      <c r="F8" s="48"/>
-      <c r="G8" s="48"/>
+      <c r="A8" s="49" t="s">
+        <v>107</v>
+      </c>
+      <c r="B8" s="49"/>
+      <c r="C8" s="49"/>
+      <c r="D8" s="49"/>
+      <c r="E8" s="49"/>
+      <c r="F8" s="49"/>
+      <c r="G8" s="49"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -4862,7 +4899,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4872,7 +4909,7 @@
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -4881,229 +4918,229 @@
       <c r="F2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="49" t="s">
-        <v>107</v>
-      </c>
-      <c r="C4" s="49"/>
-      <c r="D4" s="49"/>
-      <c r="E4" s="49"/>
-      <c r="F4" s="49"/>
+      <c r="B4" s="50" t="s">
+        <v>110</v>
+      </c>
+      <c r="C4" s="50"/>
+      <c r="D4" s="50"/>
+      <c r="E4" s="50"/>
+      <c r="F4" s="50"/>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="50" t="s">
-        <v>108</v>
-      </c>
-      <c r="C5" s="51" t="s">
-        <v>109</v>
-      </c>
-      <c r="D5" s="51"/>
-      <c r="E5" s="51"/>
-      <c r="F5" s="51"/>
+      <c r="B5" s="51" t="s">
+        <v>111</v>
+      </c>
+      <c r="C5" s="52" t="s">
+        <v>112</v>
+      </c>
+      <c r="D5" s="52"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
     </row>
     <row r="6" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="50" t="s">
-        <v>110</v>
-      </c>
-      <c r="C6" s="51" t="s">
-        <v>111</v>
-      </c>
-      <c r="D6" s="51"/>
-      <c r="E6" s="51"/>
-      <c r="F6" s="51"/>
+      <c r="B6" s="51" t="s">
+        <v>113</v>
+      </c>
+      <c r="C6" s="52" t="s">
+        <v>114</v>
+      </c>
+      <c r="D6" s="52"/>
+      <c r="E6" s="52"/>
+      <c r="F6" s="52"/>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="50" t="s">
-        <v>112</v>
-      </c>
-      <c r="C7" s="51" t="s">
-        <v>113</v>
-      </c>
-      <c r="D7" s="51"/>
-      <c r="E7" s="51"/>
-      <c r="F7" s="51"/>
+      <c r="B7" s="51" t="s">
+        <v>115</v>
+      </c>
+      <c r="C7" s="52" t="s">
+        <v>116</v>
+      </c>
+      <c r="D7" s="52"/>
+      <c r="E7" s="52"/>
+      <c r="F7" s="52"/>
     </row>
     <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="50" t="s">
-        <v>114</v>
-      </c>
-      <c r="C8" s="51" t="s">
-        <v>115</v>
-      </c>
-      <c r="D8" s="51"/>
-      <c r="E8" s="51"/>
-      <c r="F8" s="51"/>
+      <c r="B8" s="51" t="s">
+        <v>117</v>
+      </c>
+      <c r="C8" s="52" t="s">
+        <v>118</v>
+      </c>
+      <c r="D8" s="52"/>
+      <c r="E8" s="52"/>
+      <c r="F8" s="52"/>
     </row>
     <row r="9" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="49" t="s">
-        <v>116</v>
-      </c>
-      <c r="C9" s="49"/>
-      <c r="D9" s="49"/>
-      <c r="E9" s="49"/>
-      <c r="F9" s="49"/>
+      <c r="B9" s="50" t="s">
+        <v>119</v>
+      </c>
+      <c r="C9" s="50"/>
+      <c r="D9" s="50"/>
+      <c r="E9" s="50"/>
+      <c r="F9" s="50"/>
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="52" t="s">
-        <v>117</v>
-      </c>
-      <c r="C10" s="51" t="s">
-        <v>118</v>
-      </c>
-      <c r="D10" s="51"/>
-      <c r="E10" s="51"/>
-      <c r="F10" s="51"/>
+      <c r="B10" s="53" t="s">
+        <v>120</v>
+      </c>
+      <c r="C10" s="52" t="s">
+        <v>121</v>
+      </c>
+      <c r="D10" s="52"/>
+      <c r="E10" s="52"/>
+      <c r="F10" s="52"/>
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="53" t="s">
-        <v>119</v>
-      </c>
-      <c r="C11" s="51" t="s">
-        <v>120</v>
-      </c>
-      <c r="D11" s="51"/>
-      <c r="E11" s="51"/>
-      <c r="F11" s="51"/>
+      <c r="B11" s="54" t="s">
+        <v>122</v>
+      </c>
+      <c r="C11" s="52" t="s">
+        <v>123</v>
+      </c>
+      <c r="D11" s="52"/>
+      <c r="E11" s="52"/>
+      <c r="F11" s="52"/>
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="54" t="s">
-        <v>121</v>
-      </c>
-      <c r="C12" s="51" t="s">
-        <v>122</v>
-      </c>
-      <c r="D12" s="51"/>
-      <c r="E12" s="51"/>
-      <c r="F12" s="51"/>
+      <c r="B12" s="55" t="s">
+        <v>124</v>
+      </c>
+      <c r="C12" s="52" t="s">
+        <v>125</v>
+      </c>
+      <c r="D12" s="52"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="52"/>
     </row>
     <row r="13" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B13" s="49" t="s">
-        <v>123</v>
-      </c>
-      <c r="C13" s="49"/>
-      <c r="D13" s="49"/>
-      <c r="E13" s="49"/>
-      <c r="F13" s="49"/>
+      <c r="B13" s="50" t="s">
+        <v>126</v>
+      </c>
+      <c r="C13" s="50"/>
+      <c r="D13" s="50"/>
+      <c r="E13" s="50"/>
+      <c r="F13" s="50"/>
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B14" s="55" t="s">
+      <c r="B14" s="56" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="51" t="s">
-        <v>124</v>
-      </c>
-      <c r="D14" s="51"/>
-      <c r="E14" s="51"/>
-      <c r="F14" s="51"/>
+      <c r="C14" s="52" t="s">
+        <v>127</v>
+      </c>
+      <c r="D14" s="52"/>
+      <c r="E14" s="52"/>
+      <c r="F14" s="52"/>
     </row>
     <row r="15" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B15" s="56" t="s">
+      <c r="B15" s="57" t="s">
         <v>36</v>
       </c>
-      <c r="C15" s="51" t="s">
-        <v>125</v>
-      </c>
-      <c r="D15" s="51"/>
-      <c r="E15" s="51"/>
-      <c r="F15" s="51"/>
+      <c r="C15" s="52" t="s">
+        <v>128</v>
+      </c>
+      <c r="D15" s="52"/>
+      <c r="E15" s="52"/>
+      <c r="F15" s="52"/>
     </row>
     <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B16" s="57" t="s">
+      <c r="B16" s="58" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="51" t="s">
-        <v>126</v>
-      </c>
-      <c r="D16" s="51"/>
-      <c r="E16" s="51"/>
-      <c r="F16" s="51"/>
+      <c r="C16" s="52" t="s">
+        <v>129</v>
+      </c>
+      <c r="D16" s="52"/>
+      <c r="E16" s="52"/>
+      <c r="F16" s="52"/>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B17" s="58" t="s">
+      <c r="B17" s="59" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="51" t="s">
-        <v>127</v>
-      </c>
-      <c r="D17" s="51"/>
-      <c r="E17" s="51"/>
-      <c r="F17" s="51"/>
+      <c r="C17" s="52" t="s">
+        <v>130</v>
+      </c>
+      <c r="D17" s="52"/>
+      <c r="E17" s="52"/>
+      <c r="F17" s="52"/>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B18" s="59" t="s">
-        <v>128</v>
-      </c>
-      <c r="C18" s="51" t="s">
-        <v>129</v>
-      </c>
-      <c r="D18" s="51"/>
-      <c r="E18" s="51"/>
-      <c r="F18" s="51"/>
+      <c r="B18" s="60" t="s">
+        <v>131</v>
+      </c>
+      <c r="C18" s="52" t="s">
+        <v>132</v>
+      </c>
+      <c r="D18" s="52"/>
+      <c r="E18" s="52"/>
+      <c r="F18" s="52"/>
     </row>
     <row r="19" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B19" s="49" t="s">
-        <v>130</v>
-      </c>
-      <c r="C19" s="49"/>
-      <c r="D19" s="49"/>
-      <c r="E19" s="49"/>
-      <c r="F19" s="49"/>
+      <c r="B19" s="50" t="s">
+        <v>133</v>
+      </c>
+      <c r="C19" s="50"/>
+      <c r="D19" s="50"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="50"/>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B20" s="60" t="s">
-        <v>131</v>
-      </c>
-      <c r="C20" s="51" t="s">
-        <v>132</v>
-      </c>
-      <c r="D20" s="51"/>
-      <c r="E20" s="51"/>
-      <c r="F20" s="51"/>
+      <c r="B20" s="61" t="s">
+        <v>134</v>
+      </c>
+      <c r="C20" s="52" t="s">
+        <v>135</v>
+      </c>
+      <c r="D20" s="52"/>
+      <c r="E20" s="52"/>
+      <c r="F20" s="52"/>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="60" t="s">
-        <v>133</v>
-      </c>
-      <c r="C21" s="51" t="s">
-        <v>134</v>
-      </c>
-      <c r="D21" s="51"/>
-      <c r="E21" s="51"/>
-      <c r="F21" s="51"/>
+      <c r="B21" s="61" t="s">
+        <v>136</v>
+      </c>
+      <c r="C21" s="52" t="s">
+        <v>137</v>
+      </c>
+      <c r="D21" s="52"/>
+      <c r="E21" s="52"/>
+      <c r="F21" s="52"/>
     </row>
     <row r="22" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B22" s="49" t="s">
-        <v>135</v>
-      </c>
-      <c r="C22" s="49"/>
-      <c r="D22" s="49"/>
-      <c r="E22" s="49"/>
-      <c r="F22" s="49"/>
+      <c r="B22" s="50" t="s">
+        <v>138</v>
+      </c>
+      <c r="C22" s="50"/>
+      <c r="D22" s="50"/>
+      <c r="E22" s="50"/>
+      <c r="F22" s="50"/>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B23" s="50" t="s">
-        <v>136</v>
-      </c>
-      <c r="C23" s="51" t="s">
-        <v>137</v>
-      </c>
-      <c r="D23" s="51"/>
-      <c r="E23" s="51"/>
-      <c r="F23" s="51"/>
+      <c r="B23" s="51" t="s">
+        <v>139</v>
+      </c>
+      <c r="C23" s="52" t="s">
+        <v>140</v>
+      </c>
+      <c r="D23" s="52"/>
+      <c r="E23" s="52"/>
+      <c r="F23" s="52"/>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B24" s="50" t="s">
-        <v>138</v>
-      </c>
-      <c r="C24" s="51" t="s">
-        <v>139</v>
-      </c>
-      <c r="D24" s="51"/>
-      <c r="E24" s="51"/>
-      <c r="F24" s="51"/>
+      <c r="B24" s="51" t="s">
+        <v>141</v>
+      </c>
+      <c r="C24" s="52" t="s">
+        <v>142</v>
+      </c>
+      <c r="D24" s="52"/>
+      <c r="E24" s="52"/>
+      <c r="F24" s="52"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="18" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C26" s="18"/>
       <c r="D26" s="18"/>

</xml_diff>